<commit_message>
Rename domain model for PLURALISMO fake news
</commit_message>
<xml_diff>
--- a/input/FAKENEWS_BASELINE.xlsx
+++ b/input/FAKENEWS_BASELINE.xlsx
@@ -8,9 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuration" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Markets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buyers" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MarketQuota" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NewsSources" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SNSUsers" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SourceReach" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -512,7 +512,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MARKET_QUOTA</t>
+          <t>SOURCE_REACH</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -562,7 +562,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SAVED_SALES_PER_MARKET</t>
+          <t>SAVED_REPOSTS_PER_SOURCE</t>
         </is>
       </c>
       <c r="B15" t="n">

</xml_diff>

<commit_message>
Translate level labels to English
</commit_message>
<xml_diff>
--- a/input/FAKENEWS_BASELINE.xlsx
+++ b/input/FAKENEWS_BASELINE.xlsx
@@ -645,42 +645,42 @@
     <row r="3">
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bajo</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Bajo</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Bajo</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Bajo</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>High</t>
         </is>
       </c>
     </row>

</xml_diff>